<commit_message>
Forward records through 2026-10-16; ignore the PIT calibration files
Swing scans and picks, momentum picks and the watch list as recorded by the
daily jobs. The survivorship-free picker/results calibrations are
regenerable, like their non-PIT siblings, so they are ignored.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/history/momentum_picks.xlsx
+++ b/history/momentum_picks.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -15,7 +15,20 @@
   <sheets>
     <sheet name="Oct 2026" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>